<commit_message>
agilent, welco, electrolux.py all work perfectly
</commit_message>
<xml_diff>
--- a/examples/Welco/ใบสั่งงาน WELCO_P3-16-2-WI6.xlsx
+++ b/examples/Welco/ใบสั่งงาน WELCO_P3-16-2-WI6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ffa44234d445c58/Contract mfg/Welco project/ใบสั่งงาน/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vatska\software\examples\Welco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="8_{6CF77A25-100F-4229-AB49-63F0C8413D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C707D0CE-CC14-4595-B21E-65F966D8292A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD67CC6A-962C-45C5-84BC-4DC770F825C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="898" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="898" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A1_ใบสั่งงาน" sheetId="32" r:id="rId1"/>
@@ -1023,66 +1023,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1103,6 +1043,66 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1133,9 +1133,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>5603</xdr:colOff>
+      <xdr:colOff>7508</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>733985</xdr:rowOff>
+      <xdr:rowOff>735890</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3351,11 +3351,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="A1_ใบสั่งงาน"/>
       <sheetName val="A2_QC ถุงเล็ก"/>
@@ -3659,30 +3656,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M38"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="11.59765625" style="26" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" style="26" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" style="26" customWidth="1"/>
     <col min="3" max="3" width="12" style="26" customWidth="1"/>
-    <col min="4" max="4" width="15.1328125" style="45" customWidth="1"/>
-    <col min="5" max="5" width="11.796875" style="45" customWidth="1"/>
-    <col min="6" max="6" width="14.46484375" style="26" customWidth="1"/>
-    <col min="7" max="7" width="16.59765625" style="26" customWidth="1"/>
-    <col min="8" max="8" width="16.19921875" style="26" customWidth="1"/>
-    <col min="9" max="16384" width="8.73046875" style="26"/>
+    <col min="4" max="4" width="15.109375" style="45" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" style="45" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" style="26" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" style="26" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" style="26" customWidth="1"/>
+    <col min="9" max="16384" width="8.77734375" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="69.599999999999994" customHeight="1">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="102" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="103"/>
-      <c r="D1" s="103"/>
-      <c r="E1" s="103"/>
-      <c r="F1" s="103"/>
-      <c r="G1" s="103"/>
-      <c r="H1" s="103"/>
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="102"/>
     </row>
     <row r="2" spans="1:13" ht="6.6" customHeight="1">
       <c r="A2" s="24"/>
@@ -3695,14 +3692,14 @@
       <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:13" ht="28.5" customHeight="1">
-      <c r="A3" s="105" t="s">
+      <c r="A3" s="103" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="105"/>
-      <c r="C3" s="105"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="105"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
       <c r="G3" s="54" t="s">
         <v>104</v>
       </c>
@@ -3710,7 +3707,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="50" customFormat="1" ht="27.95" customHeight="1">
+    <row r="4" spans="1:13" s="50" customFormat="1" ht="27.9" customHeight="1">
       <c r="A4" s="55" t="s">
         <v>92</v>
       </c>
@@ -3724,7 +3721,7 @@
       </c>
       <c r="H4" s="58"/>
     </row>
-    <row r="5" spans="1:13" s="50" customFormat="1" ht="32.450000000000003" customHeight="1">
+    <row r="5" spans="1:13" s="50" customFormat="1" ht="32.4" customHeight="1">
       <c r="A5" s="55" t="s">
         <v>93</v>
       </c>
@@ -3750,7 +3747,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="51" customFormat="1" ht="21.95" customHeight="1">
+    <row r="7" spans="1:13" s="51" customFormat="1" ht="21.9" customHeight="1">
       <c r="A7" s="71" t="s">
         <v>38</v>
       </c>
@@ -3764,7 +3761,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="6.95" customHeight="1">
+    <row r="8" spans="1:13" ht="25.2" customHeight="1">
       <c r="A8" s="14"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -3808,24 +3805,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="50" customFormat="1" ht="25.9">
-      <c r="A10" s="110">
+    <row r="10" spans="1:13" s="50" customFormat="1" ht="25.8">
+      <c r="A10" s="90">
         <v>1</v>
       </c>
-      <c r="B10" s="111" t="s">
+      <c r="B10" s="91" t="s">
         <v>117</v>
       </c>
-      <c r="C10" s="111"/>
-      <c r="D10" s="112">
+      <c r="C10" s="91"/>
+      <c r="D10" s="92">
         <f>H6*H7/304.8/50</f>
         <v>46.587926509186353</v>
       </c>
-      <c r="E10" s="113"/>
-      <c r="F10" s="114"/>
-      <c r="G10" s="113" t="s">
+      <c r="E10" s="93"/>
+      <c r="F10" s="94"/>
+      <c r="G10" s="93" t="s">
         <v>98</v>
       </c>
-      <c r="H10" s="112">
+      <c r="H10" s="92">
         <f>50*25.4*12/H7*ROUNDUP(D10,0)</f>
         <v>5044.2253521126759</v>
       </c>
@@ -3839,17 +3836,17 @@
     </row>
     <row r="11" spans="1:13" s="50" customFormat="1" ht="16.5" customHeight="1">
       <c r="A11" s="69"/>
-      <c r="B11" s="115" t="s">
+      <c r="B11" s="95" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="116"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="119"/>
-      <c r="G11" s="118"/>
-      <c r="H11" s="117"/>
-    </row>
-    <row r="12" spans="1:13" s="50" customFormat="1" ht="25.9">
+      <c r="C11" s="96"/>
+      <c r="D11" s="97"/>
+      <c r="E11" s="98"/>
+      <c r="F11" s="99"/>
+      <c r="G11" s="98"/>
+      <c r="H11" s="97"/>
+    </row>
+    <row r="12" spans="1:13" s="50" customFormat="1" ht="25.8">
       <c r="A12" s="65">
         <v>2</v>
       </c>
@@ -3873,7 +3870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="50" customFormat="1" ht="25.9">
+    <row r="13" spans="1:13" s="50" customFormat="1" ht="25.8">
       <c r="A13" s="65">
         <v>3</v>
       </c>
@@ -3894,7 +3891,7 @@
       </c>
       <c r="H13" s="67"/>
     </row>
-    <row r="14" spans="1:13" ht="5.45" customHeight="1">
+    <row r="14" spans="1:13" ht="5.4" customHeight="1">
       <c r="A14" s="14"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
@@ -3904,7 +3901,7 @@
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
     </row>
-    <row r="15" spans="1:13" ht="23.25">
+    <row r="15" spans="1:13" ht="23.4">
       <c r="A15" s="23" t="s">
         <v>36</v>
       </c>
@@ -3916,7 +3913,7 @@
       <c r="G15" s="15"/>
       <c r="H15" s="15"/>
     </row>
-    <row r="16" spans="1:13" s="50" customFormat="1" ht="68.45" customHeight="1">
+    <row r="16" spans="1:13" s="50" customFormat="1" ht="68.400000000000006" customHeight="1">
       <c r="A16" s="63" t="s">
         <v>18</v>
       </c>
@@ -3935,12 +3932,12 @@
       <c r="F16" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="104" t="s">
+      <c r="G16" s="101" t="s">
         <v>55</v>
       </c>
-      <c r="H16" s="104"/>
-    </row>
-    <row r="17" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="H16" s="101"/>
+    </row>
+    <row r="17" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A17" s="69">
         <v>1</v>
       </c>
@@ -3955,10 +3952,10 @@
       </c>
       <c r="E17" s="70"/>
       <c r="F17" s="70"/>
-      <c r="G17" s="102"/>
-      <c r="H17" s="102"/>
-    </row>
-    <row r="18" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G17" s="100"/>
+      <c r="H17" s="100"/>
+    </row>
+    <row r="18" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A18" s="65">
         <v>2</v>
       </c>
@@ -3973,10 +3970,10 @@
       </c>
       <c r="E18" s="66"/>
       <c r="F18" s="66"/>
-      <c r="G18" s="102"/>
-      <c r="H18" s="102"/>
-    </row>
-    <row r="19" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G18" s="100"/>
+      <c r="H18" s="100"/>
+    </row>
+    <row r="19" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A19" s="65">
         <v>3</v>
       </c>
@@ -3991,10 +3988,10 @@
       </c>
       <c r="E19" s="66"/>
       <c r="F19" s="66"/>
-      <c r="G19" s="102"/>
-      <c r="H19" s="102"/>
-    </row>
-    <row r="20" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G19" s="100"/>
+      <c r="H19" s="100"/>
+    </row>
+    <row r="20" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A20" s="65">
         <v>4</v>
       </c>
@@ -4009,10 +4006,10 @@
       </c>
       <c r="E20" s="66"/>
       <c r="F20" s="66"/>
-      <c r="G20" s="102"/>
-      <c r="H20" s="102"/>
-    </row>
-    <row r="21" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G20" s="100"/>
+      <c r="H20" s="100"/>
+    </row>
+    <row r="21" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A21" s="65">
         <v>5</v>
       </c>
@@ -4027,10 +4024,10 @@
       </c>
       <c r="E21" s="66"/>
       <c r="F21" s="66"/>
-      <c r="G21" s="102"/>
-      <c r="H21" s="102"/>
-    </row>
-    <row r="22" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G21" s="100"/>
+      <c r="H21" s="100"/>
+    </row>
+    <row r="22" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A22" s="65">
         <v>6</v>
       </c>
@@ -4045,15 +4042,15 @@
       </c>
       <c r="E22" s="66"/>
       <c r="F22" s="66"/>
-      <c r="G22" s="102"/>
-      <c r="H22" s="102"/>
+      <c r="G22" s="100"/>
+      <c r="H22" s="100"/>
     </row>
     <row r="23" spans="1:8" s="50" customFormat="1" ht="5.0999999999999996" customHeight="1">
       <c r="A23" s="56"/>
       <c r="D23" s="56"/>
       <c r="E23" s="56"/>
     </row>
-    <row r="24" spans="1:8" s="50" customFormat="1" ht="25.9">
+    <row r="24" spans="1:8" s="50" customFormat="1" ht="26.4">
       <c r="A24" s="61" t="s">
         <v>37</v>
       </c>
@@ -4079,12 +4076,12 @@
       <c r="F25" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="G25" s="104" t="s">
+      <c r="G25" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H25" s="104"/>
-    </row>
-    <row r="26" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="H25" s="101"/>
+    </row>
+    <row r="26" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A26" s="69">
         <v>1</v>
       </c>
@@ -4099,10 +4096,10 @@
       </c>
       <c r="E26" s="69"/>
       <c r="F26" s="70"/>
-      <c r="G26" s="102"/>
-      <c r="H26" s="102"/>
-    </row>
-    <row r="27" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G26" s="100"/>
+      <c r="H26" s="100"/>
+    </row>
+    <row r="27" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A27" s="65">
         <v>2</v>
       </c>
@@ -4117,10 +4114,10 @@
       </c>
       <c r="E27" s="65"/>
       <c r="F27" s="66"/>
-      <c r="G27" s="102"/>
-      <c r="H27" s="102"/>
-    </row>
-    <row r="28" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G27" s="100"/>
+      <c r="H27" s="100"/>
+    </row>
+    <row r="28" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A28" s="65">
         <v>3</v>
       </c>
@@ -4135,10 +4132,10 @@
       </c>
       <c r="E28" s="65"/>
       <c r="F28" s="66"/>
-      <c r="G28" s="102"/>
-      <c r="H28" s="102"/>
-    </row>
-    <row r="29" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G28" s="100"/>
+      <c r="H28" s="100"/>
+    </row>
+    <row r="29" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A29" s="65">
         <v>4</v>
       </c>
@@ -4153,10 +4150,10 @@
       </c>
       <c r="E29" s="65"/>
       <c r="F29" s="66"/>
-      <c r="G29" s="102"/>
-      <c r="H29" s="102"/>
-    </row>
-    <row r="30" spans="1:8" s="50" customFormat="1" ht="25.9">
+      <c r="G29" s="100"/>
+      <c r="H29" s="100"/>
+    </row>
+    <row r="30" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A30" s="65">
         <v>5</v>
       </c>
@@ -4171,15 +4168,15 @@
       </c>
       <c r="E30" s="65"/>
       <c r="F30" s="66"/>
-      <c r="G30" s="102"/>
-      <c r="H30" s="102"/>
-    </row>
-    <row r="31" spans="1:8" s="50" customFormat="1" ht="9.9499999999999993" customHeight="1">
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+    </row>
+    <row r="31" spans="1:8" s="50" customFormat="1" ht="9.9" customHeight="1">
       <c r="A31" s="56"/>
       <c r="D31" s="56"/>
       <c r="E31" s="56"/>
     </row>
-    <row r="32" spans="1:8" s="50" customFormat="1" ht="25.9">
+    <row r="32" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A32" s="55" t="s">
         <v>24</v>
       </c>
@@ -4216,7 +4213,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:7" s="50" customFormat="1" ht="25.9">
+    <row r="35" spans="1:7" s="50" customFormat="1" ht="25.8">
       <c r="A35" s="56" t="s">
         <v>28</v>
       </c>
@@ -4253,6 +4250,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="G29:H29"/>
     <mergeCell ref="G30:H30"/>
@@ -4262,12 +4265,6 @@
     <mergeCell ref="G25:H25"/>
     <mergeCell ref="G26:H26"/>
     <mergeCell ref="G27:H27"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.118110236220472" right="0" top="0.118110236220472" bottom="0" header="0.118110236220472" footer="0"/>
@@ -4282,16 +4279,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D13C98-8D80-45E0-A734-2D707A643238}">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.73046875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="72.59765625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="40.59765625" style="36" customWidth="1"/>
+    <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="72.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="40.5546875" style="36" customWidth="1"/>
     <col min="4" max="4" width="17" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.59765625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1328125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="23.59765625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.73046875" style="1"/>
+    <col min="5" max="5" width="13.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4311,7 +4308,7 @@
       </c>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:7" ht="20.45" customHeight="1"/>
+    <row r="4" spans="1:7" ht="20.399999999999999" customHeight="1"/>
     <row r="5" spans="1:7" ht="37.5" customHeight="1">
       <c r="A5" s="77" t="s">
         <v>108</v>
@@ -4367,7 +4364,7 @@
         <v>P-3/16-2-WI6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="14.45" customHeight="1"/>
+    <row r="9" spans="1:7" ht="14.4" customHeight="1"/>
     <row r="10" spans="1:7" s="41" customFormat="1" ht="47.1" customHeight="1">
       <c r="A10" s="83" t="s">
         <v>72</v>
@@ -4391,11 +4388,11 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="140.44999999999999" customHeight="1">
-      <c r="A11" s="106" t="s">
+    <row r="11" spans="1:7" ht="140.4" customHeight="1">
+      <c r="A11" s="104" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="101"/>
+      <c r="B11" s="105"/>
       <c r="C11" s="42" t="s">
         <v>88</v>
       </c>
@@ -4404,9 +4401,9 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
     </row>
-    <row r="12" spans="1:7" ht="37.15" customHeight="1">
-      <c r="A12" s="106"/>
-      <c r="B12" s="101"/>
+    <row r="12" spans="1:7" ht="37.200000000000003" customHeight="1">
+      <c r="A12" s="104"/>
+      <c r="B12" s="105"/>
       <c r="C12" s="47" t="s">
         <v>65</v>
       </c>
@@ -4415,7 +4412,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
     </row>
-    <row r="13" spans="1:7" ht="194.45" customHeight="1">
+    <row r="13" spans="1:7" ht="194.4" customHeight="1">
       <c r="A13" s="48" t="s">
         <v>60</v>
       </c>
@@ -4429,7 +4426,7 @@
       <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" ht="151.5" customHeight="1">
-      <c r="A14" s="107" t="s">
+      <c r="A14" s="106" t="s">
         <v>2</v>
       </c>
       <c r="B14" s="6"/>
@@ -4441,8 +4438,8 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" ht="119.45" customHeight="1">
-      <c r="A15" s="108"/>
+    <row r="15" spans="1:7" ht="119.4" customHeight="1">
+      <c r="A15" s="107"/>
       <c r="B15" s="6"/>
       <c r="C15" s="43" t="s">
         <v>68</v>
@@ -4452,8 +4449,8 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:7" ht="122.45" customHeight="1">
-      <c r="A16" s="108" t="s">
+    <row r="16" spans="1:7" ht="122.4" customHeight="1">
+      <c r="A16" s="107" t="s">
         <v>2</v>
       </c>
       <c r="B16" s="6"/>
@@ -4465,8 +4462,8 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" ht="93.95" customHeight="1">
-      <c r="A17" s="108"/>
+    <row r="17" spans="1:7" ht="93.9" customHeight="1">
+      <c r="A17" s="107"/>
       <c r="B17" s="6"/>
       <c r="C17" s="43" t="s">
         <v>70</v>
@@ -4477,7 +4474,7 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" ht="82.5" customHeight="1">
-      <c r="A18" s="109"/>
+      <c r="A18" s="108"/>
       <c r="B18" s="6"/>
       <c r="C18" s="43" t="s">
         <v>89</v>
@@ -4487,7 +4484,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
     </row>
-    <row r="19" spans="1:7" ht="152.44999999999999" customHeight="1">
+    <row r="19" spans="1:7" ht="152.4" customHeight="1">
       <c r="A19" s="21" t="s">
         <v>30</v>
       </c>
@@ -4500,7 +4497,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="21" spans="1:7" ht="12.95" customHeight="1">
+    <row r="21" spans="1:7" ht="12.9" customHeight="1">
       <c r="E21" s="1" t="s">
         <v>1</v>
       </c>
@@ -4534,15 +4531,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="4.73046875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.59765625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="43.265625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="74.86328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.73046875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.73046875" style="1"/>
+    <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="43.21875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="74.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.77734375" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1">
@@ -4607,7 +4604,7 @@
       <c r="D8" s="30"/>
       <c r="E8" s="31"/>
     </row>
-    <row r="10" spans="1:6" s="4" customFormat="1" ht="13.9">
+    <row r="10" spans="1:6" s="4" customFormat="1">
       <c r="A10" s="32" t="s">
         <v>3</v>
       </c>
@@ -4627,122 +4624,122 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A11" s="99">
+    <row r="11" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A11" s="118">
         <v>1</v>
       </c>
-      <c r="B11" s="100" t="s">
+      <c r="B11" s="119" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="101"/>
+      <c r="C11" s="105"/>
       <c r="D11" s="17" t="s">
         <v>10</v>
       </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A12" s="99"/>
-      <c r="B12" s="100"/>
-      <c r="C12" s="101"/>
+    <row r="12" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A12" s="118"/>
+      <c r="B12" s="119"/>
+      <c r="C12" s="105"/>
       <c r="D12" s="17" t="s">
         <v>57</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A13" s="99"/>
-      <c r="B13" s="100"/>
-      <c r="C13" s="101"/>
+    <row r="13" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A13" s="118"/>
+      <c r="B13" s="119"/>
+      <c r="C13" s="105"/>
       <c r="D13" s="17" t="s">
         <v>58</v>
       </c>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A14" s="99"/>
-      <c r="B14" s="100"/>
-      <c r="C14" s="101"/>
+    <row r="14" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A14" s="118"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="105"/>
       <c r="D14" s="17" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A15" s="90">
+    <row r="15" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A15" s="109">
         <v>2</v>
       </c>
-      <c r="B15" s="93" t="s">
+      <c r="B15" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="96"/>
+      <c r="C15" s="115"/>
       <c r="D15" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A16" s="91"/>
-      <c r="B16" s="94"/>
-      <c r="C16" s="97"/>
+    <row r="16" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A16" s="110"/>
+      <c r="B16" s="113"/>
+      <c r="C16" s="116"/>
       <c r="D16" s="7" t="s">
         <v>14</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A17" s="91"/>
-      <c r="B17" s="94"/>
-      <c r="C17" s="97"/>
+    <row r="17" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A17" s="110"/>
+      <c r="B17" s="113"/>
+      <c r="C17" s="116"/>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A18" s="92"/>
-      <c r="B18" s="95"/>
-      <c r="C18" s="98"/>
+    <row r="18" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A18" s="111"/>
+      <c r="B18" s="114"/>
+      <c r="C18" s="117"/>
       <c r="D18" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A19" s="90">
+    <row r="19" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A19" s="109">
         <v>3</v>
       </c>
-      <c r="B19" s="93" t="s">
+      <c r="B19" s="112" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="96"/>
+      <c r="C19" s="115"/>
       <c r="D19" s="87" t="s">
         <v>114</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A20" s="91"/>
-      <c r="B20" s="94"/>
-      <c r="C20" s="97"/>
+    <row r="20" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A20" s="110"/>
+      <c r="B20" s="113"/>
+      <c r="C20" s="116"/>
       <c r="D20" s="11" t="s">
         <v>115</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="1:6" ht="31.9" customHeight="1">
-      <c r="A21" s="92"/>
-      <c r="B21" s="95"/>
-      <c r="C21" s="98"/>
+    <row r="21" spans="1:6" ht="31.95" customHeight="1">
+      <c r="A21" s="111"/>
+      <c r="B21" s="114"/>
+      <c r="C21" s="117"/>
       <c r="D21" s="88" t="s">
         <v>116</v>
       </c>

</xml_diff>

<commit_message>
major font changes and date format changes
</commit_message>
<xml_diff>
--- a/examples/Welco/ใบสั่งงาน WELCO_P3-16-2-WI6.xlsx
+++ b/examples/Welco/ใบสั่งงาน WELCO_P3-16-2-WI6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vatska\software\examples\Welco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD67CC6A-962C-45C5-84BC-4DC770F825C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D0660F4-CC05-4D73-A8BE-9A09F1183817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="898" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="119">
   <si>
     <t>Description</t>
   </si>
@@ -425,9 +425,6 @@
     <t>P-3/16-2-WI6</t>
   </si>
   <si>
-    <t>ASSY JOB No                                     WCA</t>
-  </si>
-  <si>
     <t>จำนวนถุงที่ตรวจสอบ / QTY</t>
   </si>
   <si>
@@ -444,6 +441,9 @@
   </si>
   <si>
     <t>ID  3/16 (4.7 mm) x OD 5/16 (7.9 mm)</t>
+  </si>
+  <si>
+    <t>ASSY JOB No</t>
   </si>
 </sst>
 </file>
@@ -816,7 +816,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1043,6 +1043,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1133,9 +1134,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>7508</xdr:colOff>
+      <xdr:colOff>20843</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>735890</xdr:rowOff>
+      <xdr:rowOff>739700</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3670,16 +3671,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="69.599999999999994" customHeight="1">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="103" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="102"/>
-      <c r="C1" s="102"/>
-      <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="102"/>
-      <c r="H1" s="102"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:13" ht="6.6" customHeight="1">
       <c r="A2" s="24"/>
@@ -3692,14 +3693,14 @@
       <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:13" ht="28.5" customHeight="1">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="104" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="103"/>
-      <c r="C3" s="103"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
       <c r="G3" s="54" t="s">
         <v>104</v>
       </c>
@@ -3730,14 +3731,20 @@
       <c r="F5" s="50" t="s">
         <v>95</v>
       </c>
-      <c r="H5" s="58"/>
+      <c r="H5" s="100">
+        <v>46244</v>
+      </c>
     </row>
     <row r="6" spans="1:13" s="50" customFormat="1" ht="27.6" customHeight="1">
       <c r="A6" s="59" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" s="60"/>
-      <c r="C6" s="58"/>
+        <v>118</v>
+      </c>
+      <c r="B6" s="60" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="58">
+        <v>1223</v>
+      </c>
       <c r="D6" s="56"/>
       <c r="E6" s="56"/>
       <c r="F6" s="50" t="s">
@@ -3810,7 +3817,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="91" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C10" s="91"/>
       <c r="D10" s="92">
@@ -3837,7 +3844,7 @@
     <row r="11" spans="1:13" s="50" customFormat="1" ht="16.5" customHeight="1">
       <c r="A11" s="69"/>
       <c r="B11" s="95" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C11" s="96"/>
       <c r="D11" s="97"/>
@@ -3932,10 +3939,10 @@
       <c r="F16" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="101" t="s">
+      <c r="G16" s="102" t="s">
         <v>55</v>
       </c>
-      <c r="H16" s="101"/>
+      <c r="H16" s="102"/>
     </row>
     <row r="17" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A17" s="69">
@@ -3952,8 +3959,8 @@
       </c>
       <c r="E17" s="70"/>
       <c r="F17" s="70"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="100"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="101"/>
     </row>
     <row r="18" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A18" s="65">
@@ -3970,8 +3977,8 @@
       </c>
       <c r="E18" s="66"/>
       <c r="F18" s="66"/>
-      <c r="G18" s="100"/>
-      <c r="H18" s="100"/>
+      <c r="G18" s="101"/>
+      <c r="H18" s="101"/>
     </row>
     <row r="19" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A19" s="65">
@@ -3988,8 +3995,8 @@
       </c>
       <c r="E19" s="66"/>
       <c r="F19" s="66"/>
-      <c r="G19" s="100"/>
-      <c r="H19" s="100"/>
+      <c r="G19" s="101"/>
+      <c r="H19" s="101"/>
     </row>
     <row r="20" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A20" s="65">
@@ -4006,8 +4013,8 @@
       </c>
       <c r="E20" s="66"/>
       <c r="F20" s="66"/>
-      <c r="G20" s="100"/>
-      <c r="H20" s="100"/>
+      <c r="G20" s="101"/>
+      <c r="H20" s="101"/>
     </row>
     <row r="21" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A21" s="65">
@@ -4024,8 +4031,8 @@
       </c>
       <c r="E21" s="66"/>
       <c r="F21" s="66"/>
-      <c r="G21" s="100"/>
-      <c r="H21" s="100"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
     </row>
     <row r="22" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A22" s="65">
@@ -4042,8 +4049,8 @@
       </c>
       <c r="E22" s="66"/>
       <c r="F22" s="66"/>
-      <c r="G22" s="100"/>
-      <c r="H22" s="100"/>
+      <c r="G22" s="101"/>
+      <c r="H22" s="101"/>
     </row>
     <row r="23" spans="1:8" s="50" customFormat="1" ht="5.0999999999999996" customHeight="1">
       <c r="A23" s="56"/>
@@ -4076,10 +4083,10 @@
       <c r="F25" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="G25" s="101" t="s">
+      <c r="G25" s="102" t="s">
         <v>56</v>
       </c>
-      <c r="H25" s="101"/>
+      <c r="H25" s="102"/>
     </row>
     <row r="26" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A26" s="69">
@@ -4096,8 +4103,8 @@
       </c>
       <c r="E26" s="69"/>
       <c r="F26" s="70"/>
-      <c r="G26" s="100"/>
-      <c r="H26" s="100"/>
+      <c r="G26" s="101"/>
+      <c r="H26" s="101"/>
     </row>
     <row r="27" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A27" s="65">
@@ -4114,8 +4121,8 @@
       </c>
       <c r="E27" s="65"/>
       <c r="F27" s="66"/>
-      <c r="G27" s="100"/>
-      <c r="H27" s="100"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
     </row>
     <row r="28" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A28" s="65">
@@ -4132,8 +4139,8 @@
       </c>
       <c r="E28" s="65"/>
       <c r="F28" s="66"/>
-      <c r="G28" s="100"/>
-      <c r="H28" s="100"/>
+      <c r="G28" s="101"/>
+      <c r="H28" s="101"/>
     </row>
     <row r="29" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A29" s="65">
@@ -4150,8 +4157,8 @@
       </c>
       <c r="E29" s="65"/>
       <c r="F29" s="66"/>
-      <c r="G29" s="100"/>
-      <c r="H29" s="100"/>
+      <c r="G29" s="101"/>
+      <c r="H29" s="101"/>
     </row>
     <row r="30" spans="1:8" s="50" customFormat="1" ht="25.8">
       <c r="A30" s="65">
@@ -4168,8 +4175,8 @@
       </c>
       <c r="E30" s="65"/>
       <c r="F30" s="66"/>
-      <c r="G30" s="100"/>
-      <c r="H30" s="100"/>
+      <c r="G30" s="101"/>
+      <c r="H30" s="101"/>
     </row>
     <row r="31" spans="1:8" s="50" customFormat="1" ht="9.9" customHeight="1">
       <c r="A31" s="56"/>
@@ -4389,10 +4396,10 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="140.4" customHeight="1">
-      <c r="A11" s="104" t="s">
+      <c r="A11" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="105"/>
+      <c r="B11" s="106"/>
       <c r="C11" s="42" t="s">
         <v>88</v>
       </c>
@@ -4402,8 +4409,8 @@
       <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:7" ht="37.200000000000003" customHeight="1">
-      <c r="A12" s="104"/>
-      <c r="B12" s="105"/>
+      <c r="A12" s="105"/>
+      <c r="B12" s="106"/>
       <c r="C12" s="47" t="s">
         <v>65</v>
       </c>
@@ -4426,7 +4433,7 @@
       <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" ht="151.5" customHeight="1">
-      <c r="A14" s="106" t="s">
+      <c r="A14" s="107" t="s">
         <v>2</v>
       </c>
       <c r="B14" s="6"/>
@@ -4439,7 +4446,7 @@
       <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:7" ht="119.4" customHeight="1">
-      <c r="A15" s="107"/>
+      <c r="A15" s="108"/>
       <c r="B15" s="6"/>
       <c r="C15" s="43" t="s">
         <v>68</v>
@@ -4450,7 +4457,7 @@
       <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:7" ht="122.4" customHeight="1">
-      <c r="A16" s="107" t="s">
+      <c r="A16" s="108" t="s">
         <v>2</v>
       </c>
       <c r="B16" s="6"/>
@@ -4463,7 +4470,7 @@
       <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:7" ht="93.9" customHeight="1">
-      <c r="A17" s="107"/>
+      <c r="A17" s="108"/>
       <c r="B17" s="6"/>
       <c r="C17" s="43" t="s">
         <v>70</v>
@@ -4474,7 +4481,7 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" ht="82.5" customHeight="1">
-      <c r="A18" s="108"/>
+      <c r="A18" s="109"/>
       <c r="B18" s="6"/>
       <c r="C18" s="43" t="s">
         <v>89</v>
@@ -4594,7 +4601,7 @@
     </row>
     <row r="8" spans="1:6" ht="21" customHeight="1">
       <c r="A8" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="86">
@@ -4625,13 +4632,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A11" s="118">
+      <c r="A11" s="119">
         <v>1</v>
       </c>
-      <c r="B11" s="119" t="s">
+      <c r="B11" s="120" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="105"/>
+      <c r="C11" s="106"/>
       <c r="D11" s="17" t="s">
         <v>10</v>
       </c>
@@ -4639,9 +4646,9 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A12" s="118"/>
-      <c r="B12" s="119"/>
-      <c r="C12" s="105"/>
+      <c r="A12" s="119"/>
+      <c r="B12" s="120"/>
+      <c r="C12" s="106"/>
       <c r="D12" s="17" t="s">
         <v>57</v>
       </c>
@@ -4649,9 +4656,9 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A13" s="118"/>
-      <c r="B13" s="119"/>
-      <c r="C13" s="105"/>
+      <c r="A13" s="119"/>
+      <c r="B13" s="120"/>
+      <c r="C13" s="106"/>
       <c r="D13" s="17" t="s">
         <v>58</v>
       </c>
@@ -4659,9 +4666,9 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A14" s="118"/>
-      <c r="B14" s="119"/>
-      <c r="C14" s="105"/>
+      <c r="A14" s="119"/>
+      <c r="B14" s="120"/>
+      <c r="C14" s="106"/>
       <c r="D14" s="17" t="s">
         <v>11</v>
       </c>
@@ -4669,13 +4676,13 @@
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A15" s="109">
+      <c r="A15" s="110">
         <v>2</v>
       </c>
-      <c r="B15" s="112" t="s">
+      <c r="B15" s="113" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="115"/>
+      <c r="C15" s="116"/>
       <c r="D15" s="7" t="s">
         <v>13</v>
       </c>
@@ -4683,9 +4690,9 @@
       <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A16" s="110"/>
-      <c r="B16" s="113"/>
-      <c r="C16" s="116"/>
+      <c r="A16" s="111"/>
+      <c r="B16" s="114"/>
+      <c r="C16" s="117"/>
       <c r="D16" s="7" t="s">
         <v>14</v>
       </c>
@@ -4693,9 +4700,9 @@
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A17" s="110"/>
-      <c r="B17" s="113"/>
-      <c r="C17" s="116"/>
+      <c r="A17" s="111"/>
+      <c r="B17" s="114"/>
+      <c r="C17" s="117"/>
       <c r="D17" s="7" t="s">
         <v>33</v>
       </c>
@@ -4703,9 +4710,9 @@
       <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A18" s="111"/>
-      <c r="B18" s="114"/>
-      <c r="C18" s="117"/>
+      <c r="A18" s="112"/>
+      <c r="B18" s="115"/>
+      <c r="C18" s="118"/>
       <c r="D18" s="7" t="s">
         <v>12</v>
       </c>
@@ -4713,35 +4720,35 @@
       <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A19" s="109">
+      <c r="A19" s="110">
         <v>3</v>
       </c>
-      <c r="B19" s="112" t="s">
+      <c r="B19" s="113" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="115"/>
+      <c r="C19" s="116"/>
       <c r="D19" s="87" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A20" s="110"/>
-      <c r="B20" s="113"/>
-      <c r="C20" s="116"/>
+      <c r="A20" s="111"/>
+      <c r="B20" s="114"/>
+      <c r="C20" s="117"/>
       <c r="D20" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A21" s="111"/>
-      <c r="B21" s="114"/>
-      <c r="C21" s="117"/>
+      <c r="A21" s="112"/>
+      <c r="B21" s="115"/>
+      <c r="C21" s="118"/>
       <c r="D21" s="88" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>

</xml_diff>